<commit_message>
test(golden): make the golden regression suite actually run
`ASSETS` resolved to ``tests/integration/assets``, which does not exist, so all
six golden comparisons skipped themselves and the suite never ran — not on CI,
not locally. Point it at ``tests/assets`` where the docstring already said the
copies live.

Two behaviours that the openpyxl object model cannot see are now compared
straight from the package as well:

- chart data references, read from every ``xl/charts/chart*.xml`` with the XML
  prefix normalised away, and
- the ``refreshOnLoad`` flag of each pivot cache.

Running the suite for the first time surfaced a stale win32com pivot golden: it
was generated before the ``RefreshOnFileOpen`` fix, so it had no
``refreshOnLoad``. Regenerated with
``uv run python scripts/fill_demo.py --output-dir tests/assets/golden``.
</commit_message>
<xml_diff>
--- a/tests/assets/golden/win32com/test_template_3_pivot_filled.xlsx
+++ b/tests/assets/golden/win32com/test_template_3_pivot_filled.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\botti\Desktop\xlfill\tests\assets\golden\win32com\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\botti\AppData\Local\Temp\golden-regen\win32com\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF2F2246-CB30-4F6C-9872-87BD0C607CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BAC3A7A-3825-4338-B4AF-376437FC54E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId3"/>
+    <pivotCache cacheId="7" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -170,6 +170,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -216,7 +217,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Harald Böttiger" refreshedDate="46215.420744907409" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="6" xr:uid="{02BCE8ED-B302-4D38-B6A4-57F051FC750D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Harald Böttiger" refreshedDate="46313.689210069446" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="6" xr:uid="{02BCE8ED-B302-4D38-B6A4-57F051FC750D}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:E7" sheet="Sales Data"/>
   </cacheSource>
@@ -301,7 +302,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1200EBB8-2765-48BF-A980-22697AC54BB1}" name="SalesPivot" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1200EBB8-2765-48BF-A980-22697AC54BB1}" name="SalesPivot" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -678,16 +679,16 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="2">
@@ -695,16 +696,16 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E3" s="2">
@@ -712,16 +713,16 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E4" s="2">
@@ -729,16 +730,16 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="2">
@@ -746,16 +747,16 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="2">
@@ -763,16 +764,16 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="2">

</xml_diff>